<commit_message>
Edit parse excel to .js
</commit_message>
<xml_diff>
--- a/layout.xlsx
+++ b/layout.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="732" uniqueCount="732">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="732" uniqueCount="731">
   <si>
     <r>
       <rPr>
@@ -2886,6 +2886,9 @@
     </r>
   </si>
   <si>
+    <t>SIGNIFICADO</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <rFont val="Arial"/>
@@ -2893,7 +2896,7 @@
         <color theme="1"/>
         <sz val="8.0"/>
       </rPr>
-      <t>SIGIFICADO</t>
+      <t>OBRIGATÓRIO</t>
     </r>
   </si>
   <si>
@@ -2904,7 +2907,7 @@
         <color theme="1"/>
         <sz val="8.0"/>
       </rPr>
-      <t>OBRIGATÓRIO</t>
+      <t>POSIÇÃO</t>
     </r>
   </si>
   <si>
@@ -2915,7 +2918,7 @@
         <color theme="1"/>
         <sz val="8.0"/>
       </rPr>
-      <t>POSIÇÃO</t>
+      <t>PICTURE</t>
     </r>
   </si>
   <si>
@@ -2926,7 +2929,255 @@
         <color theme="1"/>
         <sz val="8.0"/>
       </rPr>
-      <t>PICTURE</t>
+      <t>CONTEÚDO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>TIPO DE REGISTRO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>IDENTIFICAÇÃO DO REGISTRO TRAILER</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>SIM</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>9(01)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>BRANCOS</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>BRANCOS</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>NÃO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>X(711)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>VALOR TOTAL</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>VALOR TOTAL DOS REGISTROS</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>SIM</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>9(15)V9(2)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color rgb="FF000000"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t xml:space="preserve">SOMATÓRIA DO CAMPO VALOR ORIGINAL DO
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color rgb="FF000000"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>DETALHE</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>QTDE DE REGISTROS</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>QUANTIDADE DE REGISTROS DE TRANSAÇÃO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>SIM</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>9(15)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color rgb="FF000000"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t xml:space="preserve">SOMATÓRIA DA QUANTIDADE DE
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color rgb="FF000000"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>REGISTROS DO ARQUIVO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>NÚMERO SEQÜENCIAL</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>NÚMERO SEQÜENCIAL DO REGISTRO NO ARQUIVO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>SIM</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>9(06)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>s</t>
     </r>
   </si>
   <si>
@@ -2937,255 +3188,7 @@
         <color theme="1"/>
         <sz val="8.0"/>
       </rPr>
-      <t>CONTEÚDO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>TIPO DE REGISTRO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>IDENTIFICAÇÃO DO REGISTRO TRAILER</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>SIM</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>9(01)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>BRANCOS</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>BRANCOS</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>NÃO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>X(711)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>VALOR TOTAL</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>VALOR TOTAL DOS REGISTROS</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>SIM</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>9(15)V9(2)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color rgb="FF000000"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t xml:space="preserve">SOMATÓRIA DO CAMPO VALOR ORIGINAL DO
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color rgb="FF000000"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>DETALHE</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>QTDE DE REGISTROS</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>QUANTIDADE DE REGISTROS DE TRANSAÇÃO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>SIM</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>9(15)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color rgb="FF000000"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t xml:space="preserve">SOMATÓRIA DA QUANTIDADE DE
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color rgb="FF000000"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>REGISTROS DO ARQUIVO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>NÚMERO SEQÜENCIAL</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>NÚMERO SEQÜENCIAL DO REGISTRO NO ARQUIVO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>SIM</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>9(06)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>s</t>
+      <t>NOME DO CAMPO</t>
     </r>
   </si>
   <si>
@@ -3196,7 +3199,7 @@
         <color theme="1"/>
         <sz val="8.0"/>
       </rPr>
-      <t>NOME DO CAMPO</t>
+      <t>SIGNIFICADO</t>
     </r>
   </si>
   <si>
@@ -3207,7 +3210,7 @@
         <color theme="1"/>
         <sz val="8.0"/>
       </rPr>
-      <t>SIGNIFICADO</t>
+      <t>OBRIGATÓRIO</t>
     </r>
   </si>
   <si>
@@ -3218,7 +3221,7 @@
         <color theme="1"/>
         <sz val="8.0"/>
       </rPr>
-      <t>OBRIGATÓRIO</t>
+      <t>POSIÇÃO</t>
     </r>
   </si>
   <si>
@@ -3229,7 +3232,7 @@
         <color theme="1"/>
         <sz val="8.0"/>
       </rPr>
-      <t>POSIÇÃO</t>
+      <t>PICTURE</t>
     </r>
   </si>
   <si>
@@ -3240,7 +3243,924 @@
         <color theme="1"/>
         <sz val="8.0"/>
       </rPr>
-      <t>PICTURE</t>
+      <t>CONTEÚDO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>TIPO DE REGISTRO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>IDENTIFICAÇÃO DO REGISTRO HEADER</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>SIM</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>9(01)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>CÓDIGO DE RETORNO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>IDENTIFICAÇÃO DO ARQUIVO RETORNO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>SIM</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>9(01)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>LITERAL DE RETORNO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>IDENTIFICAÇÃO. POR EXTENSO DO TIPO DE MOVIMENTO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>SIM</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>X(07)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>RETORNO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>CÓDIGO DO SERVIÇO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>IDENTIFICAÇÃO DO TIPO DE SERVIÇO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>SIM</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>9(02)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>LITERAL DE SERVIÇO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>IDENTIFICAÇÃO POR EXTENSO DO TIPO DE SERVIÇO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>SIM</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>X(15)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>PIX</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>ISPB PARTICIPANTE</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>PSP DO USUARIO RECEBEDOR</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>SIM</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>X(08)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>Deve ser preenchido com ISPB do PSP</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>CÓDIGO DE INSCRIÇÃO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>TIPO DE INSCRIÇÃO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>SIM</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>9(02)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>NOTA 1</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>CPF CNPJ</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>CPF CNPJ DO USUARIO RECEBEDOR</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>SIM</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>9(14)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>Identificação única do usuário recebedor</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>AGÊNCIA</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>AGÊNCIA DO USUARIO RECEBEDOR</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>NÃO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>9(04)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>Agência do usuário recebedor.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>CONTA</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>CONTA USUÁRIO RECEBEDOR</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>NÃO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>9(20)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>Número da conta transacional usuário recebedor</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>TIPO CONTA</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>TIPO CONTA USUÁRIO RECEBEDOR</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>NÃO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>X(04)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>NOTA 2</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>CHAVE Pix</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>CHAVE Pix</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>NÃO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>X(77)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>NOTA 3</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>DATA DE GERAÇÃO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>DATA DE GERAÇÃO DO ARQUIVO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>SIM</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>9(08)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>AAAAMMDD</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>CÓDIGO DO CONVENIO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>CÓDIGO DO CONVENIO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>NÃO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>X(30)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>EXCLUSIVO PSP RECEBEDOR</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>EXCLUSIVO PSP RECEBEDOR</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>NÃO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>X(60)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>Campo para uso exclusivo do PSP recebedor</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>CÓDIGOS DE ERRO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>CÓDIGOS DE ERRO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>NÃO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>X(30)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>NOTA 23</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>BRANCOS</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>COMPLEMENTO DO REGISTRO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>NÃO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>X(458)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>VERSAO DO ARQUIVO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>VERSAO DO LAYOUT DO ARQUIVO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>SIM</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>9(3)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color rgb="FF000000"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t xml:space="preserve">1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color rgb="FF000000"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t xml:space="preserve">CONTEÚDO PODE SER ALTERADO DE ACORDO
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color rgb="FF000000"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>COM VERSÃO DO LAYOUT</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color rgb="FF000000"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t xml:space="preserve">NÚMERO
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color rgb="FF000000"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>SEQÜENCIAL DO ARQUIVO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>NÚMERO SEQÜENCIAL DO ARQUIVO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>SIM</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial MT"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>9(06)</t>
     </r>
   </si>
   <si>
@@ -3251,946 +4171,7 @@
         <color theme="1"/>
         <sz val="8.0"/>
       </rPr>
-      <t>CONTEÚDO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>TIPO DE REGISTRO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>IDENTIFICAÇÃO DO REGISTRO HEADER</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>SIM</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>9(01)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>CÓDIGO DE RETORNO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>IDENTIFICAÇÃO DO ARQUIVO RETORNO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>SIM</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>9(01)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>LITERAL DE RETORNO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>IDENTIFICAÇÃO. POR EXTENSO DO TIPO DE MOVIMENTO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>SIM</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>X(07)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>RETORNO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>CÓDIGO DO SERVIÇO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>IDENTIFICAÇÃO DO TIPO DE SERVIÇO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>SIM</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>9(02)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>LITERAL DE SERVIÇO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>IDENTIFICAÇÃO POR EXTENSO DO TIPO DE SERVIÇO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>SIM</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>X(15)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>PIX</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>ISPB PARTICIPANTE</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>PSP DO USUARIO RECEBEDOR</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>SIM</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>X(08)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>Deve ser preenchido com ISPB do PSP</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>CÓDIGO DE INSCRIÇÃO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>TIPO DE INSCRIÇÃO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>SIM</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>9(02)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>NOTA 1</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>CPF CNPJ</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>CPF CNPJ DO USUARIO RECEBEDOR</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>SIM</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>9(14)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>Identificação única do usuário recebedor</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>AGÊNCIA</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>AGÊNCIA DO USUARIO RECEBEDOR</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>NÃO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>9(04)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>Agência do usuário recebedor.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>CONTA</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>CONTA USUÁRIO RECEBEDOR</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>NÃO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>9(20)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>Número da conta transacional usuário recebedor</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>TIPO CONTA</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>TIPO CONTA USUÁRIO RECEBEDOR</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>NÃO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>X(04)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>NOTA 2</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>CHAVE Pix</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>CHAVE Pix</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>NÃO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>X(77)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>NOTA 3</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>DATA DE GERAÇÃO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>DATA DE GERAÇÃO DO ARQUIVO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>SIM</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>9(08)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>AAAAMMDD</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>CÓDIGO DO CONVENIO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>CÓDIGO DO CONVENIO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>NÃO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>X(30)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>EXCLUSIVO PSP RECEBEDOR</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>EXCLUSIVO PSP RECEBEDOR</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>NÃO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>X(60)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>Campo para uso exclusivo do PSP recebedor</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>CÓDIGOS DE ERRO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>CÓDIGOS DE ERRO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>NÃO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>X(30)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>NOTA 23</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>BRANCOS</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>COMPLEMENTO DO REGISTRO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>NÃO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>X(458)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>VERSAO DO ARQUIVO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>VERSAO DO LAYOUT DO ARQUIVO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>SIM</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>9(3)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color rgb="FF000000"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t xml:space="preserve">1
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color rgb="FF000000"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t xml:space="preserve">CONTEÚDO PODE SER ALTERADO DE ACORDO
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color rgb="FF000000"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>COM VERSÃO DO LAYOUT</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color rgb="FF000000"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t xml:space="preserve">NÚMERO
-</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color rgb="FF000000"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>SEQÜENCIAL DO ARQUIVO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>NÚMERO SEQÜENCIAL DO ARQUIVO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>SIM</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial MT"/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>9(06)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
       <t>NOME DO CAMPO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="8.0"/>
-      </rPr>
-      <t>SIGNIFICADO</t>
     </r>
   </si>
   <si>
@@ -7827,7 +7808,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="0"/>
     </xf>
@@ -7891,6 +7872,9 @@
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
@@ -7911,6 +7895,9 @@
     </xf>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="2" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="4" numFmtId="1" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" shrinkToFit="1" vertical="top" wrapText="0"/>
@@ -9721,40 +9708,40 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>693</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>694</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>695</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>696</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>697</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>698</v>
-      </c>
-      <c r="G1" s="30"/>
+      <c r="G1" s="32"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="s">
+        <v>698</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>699</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>700</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>701</v>
       </c>
       <c r="D2" s="6">
         <v>1001.0</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="F2" s="7">
         <v>9.0</v>
@@ -9762,19 +9749,19 @@
     </row>
     <row r="3">
       <c r="A3" s="4" t="s">
+        <v>702</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>703</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>704</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>705</v>
       </c>
       <c r="D3" s="6">
         <v>2002.0</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="F3" s="7">
         <v>2.0</v>
@@ -9782,19 +9769,19 @@
     </row>
     <row r="4">
       <c r="A4" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>707</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>708</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>709</v>
       </c>
       <c r="D4" s="6">
         <v>3004.0</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="F4" s="9">
         <v>2.0</v>
@@ -9802,93 +9789,93 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="s">
+        <v>710</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>711</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>712</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>713</v>
       </c>
       <c r="D5" s="6">
         <v>5012.0</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="F5" s="14"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="s">
+        <v>714</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>715</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>716</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>717</v>
       </c>
       <c r="D6" s="6">
         <v>13042.0</v>
       </c>
       <c r="E6" s="4" t="s">
+        <v>717</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>718</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>719</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="s">
+        <v>719</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>720</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>721</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>722</v>
       </c>
       <c r="D7" s="6">
         <v>43729.0</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="F7" s="14"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="s">
+        <v>723</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>724</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>725</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>726</v>
       </c>
       <c r="D8" s="6">
         <v>730744.0</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="F8" s="13"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="s">
+        <v>727</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>728</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>729</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>730</v>
       </c>
       <c r="D9" s="6">
         <v>745750.0</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="F9" s="13"/>
     </row>
@@ -12657,10 +12644,10 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A13:H13"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A15:H15"/>
     <mergeCell ref="A16:H16"/>
-    <mergeCell ref="A13:H13"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
@@ -12692,7 +12679,7 @@
       <c r="A1" s="1" t="s">
         <v>270</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="21" t="s">
         <v>271</v>
       </c>
       <c r="C1" s="2" t="s">
@@ -12830,7 +12817,7 @@
     <row r="30" ht="18.75" customHeight="1"/>
     <row r="31" ht="18.75" customHeight="1"/>
     <row r="32" ht="11.25" customHeight="1">
-      <c r="A32" s="21" t="s">
+      <c r="A32" s="22" t="s">
         <v>298</v>
       </c>
     </row>
@@ -13839,9 +13826,9 @@
       <c r="F1" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="s">
@@ -14225,22 +14212,22 @@
       <c r="I23" s="16"/>
     </row>
     <row r="24">
-      <c r="G24" s="23"/>
+      <c r="G24" s="24"/>
     </row>
     <row r="25">
-      <c r="G25" s="24"/>
-      <c r="I25" s="25"/>
+      <c r="G25" s="25"/>
+      <c r="I25" s="26"/>
     </row>
     <row r="26">
-      <c r="G26" s="26"/>
-      <c r="I26" s="25"/>
+      <c r="G26" s="27"/>
+      <c r="I26" s="26"/>
     </row>
     <row r="27">
-      <c r="G27" s="26"/>
-      <c r="I27" s="25"/>
+      <c r="G27" s="27"/>
+      <c r="I27" s="26"/>
     </row>
     <row r="28">
-      <c r="I28" s="27"/>
+      <c r="I28" s="28"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>
@@ -14267,651 +14254,651 @@
       <c r="A1" s="1" t="s">
         <v>394</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="29" t="s">
+        <v>271</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>397</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="17" t="s">
         <v>398</v>
-      </c>
-      <c r="F1" s="17" t="s">
-        <v>399</v>
       </c>
     </row>
     <row r="2" ht="18.75" customHeight="1">
       <c r="A2" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="B2" s="19" t="s">
         <v>400</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="C2" s="5" t="s">
         <v>401</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>402</v>
       </c>
       <c r="D2" s="6">
         <v>1001.0</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>403</v>
-      </c>
-      <c r="F2" s="28">
+        <v>402</v>
+      </c>
+      <c r="F2" s="30">
         <v>1.0</v>
       </c>
     </row>
     <row r="3" ht="27.75" customHeight="1">
       <c r="A3" s="4" t="s">
+        <v>403</v>
+      </c>
+      <c r="B3" s="19" t="s">
         <v>404</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="C3" s="5" t="s">
         <v>405</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>406</v>
       </c>
       <c r="D3" s="6">
         <v>2009.0</v>
       </c>
       <c r="E3" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="F3" s="19" t="s">
         <v>407</v>
-      </c>
-      <c r="F3" s="19" t="s">
-        <v>408</v>
       </c>
     </row>
     <row r="4" ht="18.75" customHeight="1">
       <c r="A4" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="B4" s="19" t="s">
         <v>409</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="C4" s="5" t="s">
         <v>410</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>411</v>
       </c>
       <c r="D4" s="6">
         <v>10011.0</v>
       </c>
       <c r="E4" s="4" t="s">
+        <v>411</v>
+      </c>
+      <c r="F4" s="19" t="s">
         <v>412</v>
-      </c>
-      <c r="F4" s="19" t="s">
-        <v>413</v>
       </c>
     </row>
     <row r="5" ht="11.25" customHeight="1">
       <c r="A5" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>414</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>415</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>416</v>
       </c>
       <c r="D5" s="6">
         <v>12025.0</v>
       </c>
       <c r="E5" s="4" t="s">
+        <v>416</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>417</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>418</v>
       </c>
     </row>
     <row r="6" ht="11.25" customHeight="1">
       <c r="A6" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>419</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>420</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>421</v>
       </c>
       <c r="D6" s="6">
         <v>26029.0</v>
       </c>
       <c r="E6" s="4" t="s">
+        <v>421</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>422</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>423</v>
       </c>
     </row>
     <row r="7" ht="18.75" customHeight="1">
       <c r="A7" s="4" t="s">
+        <v>423</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>424</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>425</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>426</v>
       </c>
       <c r="D7" s="6">
         <v>30049.0</v>
       </c>
       <c r="E7" s="4" t="s">
+        <v>426</v>
+      </c>
+      <c r="F7" s="10" t="s">
         <v>427</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>428</v>
       </c>
     </row>
     <row r="8" ht="18.75" customHeight="1">
       <c r="A8" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>429</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>430</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>431</v>
       </c>
       <c r="D8" s="6">
         <v>50053.0</v>
       </c>
       <c r="E8" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="F8" s="4" t="s">
         <v>432</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>433</v>
       </c>
     </row>
     <row r="9" ht="11.25" customHeight="1">
       <c r="A9" s="4" t="s">
+        <v>433</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>434</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>435</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>436</v>
       </c>
       <c r="D9" s="6">
         <v>54130.0</v>
       </c>
       <c r="E9" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="F9" s="4" t="s">
         <v>437</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>438</v>
       </c>
     </row>
     <row r="10" ht="64.5" customHeight="1">
       <c r="A10" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>439</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="C10" s="5" t="s">
         <v>440</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>441</v>
       </c>
       <c r="D10" s="6">
         <v>131131.0</v>
       </c>
       <c r="E10" s="4" t="s">
+        <v>441</v>
+      </c>
+      <c r="F10" s="4" t="s">
         <v>442</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>443</v>
       </c>
     </row>
     <row r="11" ht="18.75" customHeight="1">
       <c r="A11" s="4" t="s">
+        <v>443</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>444</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="C11" s="5" t="s">
         <v>445</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>446</v>
       </c>
       <c r="D11" s="6">
         <v>132133.0</v>
       </c>
       <c r="E11" s="4" t="s">
+        <v>446</v>
+      </c>
+      <c r="F11" s="4" t="s">
         <v>447</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>448</v>
       </c>
     </row>
     <row r="12" ht="36.75" customHeight="1">
       <c r="A12" s="4" t="s">
+        <v>448</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>449</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="C12" s="5" t="s">
         <v>450</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>451</v>
       </c>
       <c r="D12" s="6">
         <v>134141.0</v>
       </c>
       <c r="E12" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="F12" s="4" t="s">
         <v>452</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>453</v>
       </c>
     </row>
     <row r="13" ht="18.75" customHeight="1">
       <c r="A13" s="4" t="s">
+        <v>453</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>454</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="C13" s="5" t="s">
         <v>455</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>456</v>
       </c>
       <c r="D13" s="6">
         <v>142176.0</v>
       </c>
       <c r="E13" s="4" t="s">
+        <v>456</v>
+      </c>
+      <c r="F13" s="4" t="s">
         <v>457</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>458</v>
       </c>
     </row>
     <row r="14" ht="18.75" customHeight="1">
       <c r="A14" s="4" t="s">
+        <v>458</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>459</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="C14" s="5" t="s">
         <v>460</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>461</v>
       </c>
       <c r="D14" s="6">
         <v>177191.0</v>
       </c>
       <c r="E14" s="4" t="s">
+        <v>461</v>
+      </c>
+      <c r="F14" s="10" t="s">
         <v>462</v>
-      </c>
-      <c r="F14" s="10" t="s">
-        <v>463</v>
       </c>
     </row>
     <row r="15" ht="18.75" customHeight="1">
       <c r="A15" s="4" t="s">
+        <v>463</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>464</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="C15" s="5" t="s">
         <v>465</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>466</v>
       </c>
       <c r="D15" s="6">
         <v>192199.0</v>
       </c>
       <c r="E15" s="4" t="s">
+        <v>466</v>
+      </c>
+      <c r="F15" s="4" t="s">
         <v>467</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>468</v>
       </c>
     </row>
     <row r="16" ht="27.75" customHeight="1">
       <c r="A16" s="4" t="s">
+        <v>468</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>469</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="C16" s="5" t="s">
         <v>470</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>471</v>
       </c>
       <c r="D16" s="6">
         <v>200216.0</v>
       </c>
       <c r="E16" s="4" t="s">
+        <v>471</v>
+      </c>
+      <c r="F16" s="10" t="s">
         <v>472</v>
-      </c>
-      <c r="F16" s="10" t="s">
-        <v>473</v>
       </c>
     </row>
     <row r="17" ht="18.75" customHeight="1">
       <c r="A17" s="4" t="s">
+        <v>473</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>474</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="C17" s="5" t="s">
         <v>475</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>476</v>
       </c>
       <c r="D17" s="6">
         <v>217233.0</v>
       </c>
       <c r="E17" s="4" t="s">
+        <v>476</v>
+      </c>
+      <c r="F17" s="4" t="s">
         <v>477</v>
-      </c>
-      <c r="F17" s="4" t="s">
-        <v>478</v>
       </c>
     </row>
     <row r="18" ht="18.75" customHeight="1">
       <c r="A18" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>479</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="C18" s="5" t="s">
         <v>480</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>481</v>
       </c>
       <c r="D18" s="6">
         <v>234250.0</v>
       </c>
       <c r="E18" s="4" t="s">
+        <v>481</v>
+      </c>
+      <c r="F18" s="4" t="s">
         <v>482</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>483</v>
       </c>
     </row>
     <row r="19" ht="27.75" customHeight="1">
       <c r="A19" s="4" t="s">
+        <v>483</v>
+      </c>
+      <c r="B19" s="4" t="s">
         <v>484</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="C19" s="5" t="s">
         <v>485</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>486</v>
       </c>
       <c r="D19" s="6">
         <v>251267.0</v>
       </c>
       <c r="E19" s="4" t="s">
+        <v>486</v>
+      </c>
+      <c r="F19" s="4" t="s">
         <v>487</v>
-      </c>
-      <c r="F19" s="4" t="s">
-        <v>488</v>
       </c>
     </row>
     <row r="20" ht="27.75" customHeight="1">
       <c r="A20" s="4" t="s">
+        <v>488</v>
+      </c>
+      <c r="B20" s="4" t="s">
         <v>489</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="C20" s="5" t="s">
         <v>490</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>491</v>
       </c>
       <c r="D20" s="6">
         <v>268284.0</v>
       </c>
       <c r="E20" s="4" t="s">
+        <v>491</v>
+      </c>
+      <c r="F20" s="4" t="s">
         <v>492</v>
-      </c>
-      <c r="F20" s="4" t="s">
-        <v>493</v>
       </c>
     </row>
     <row r="21" ht="27.75" customHeight="1">
       <c r="A21" s="4" t="s">
+        <v>493</v>
+      </c>
+      <c r="B21" s="4" t="s">
         <v>494</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="C21" s="5" t="s">
         <v>495</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>496</v>
       </c>
       <c r="D21" s="6">
         <v>285301.0</v>
       </c>
       <c r="E21" s="4" t="s">
+        <v>496</v>
+      </c>
+      <c r="F21" s="4" t="s">
         <v>497</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>498</v>
       </c>
     </row>
     <row r="22" ht="27.75" customHeight="1">
       <c r="A22" s="4" t="s">
+        <v>498</v>
+      </c>
+      <c r="B22" s="4" t="s">
         <v>499</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="C22" s="5" t="s">
         <v>500</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>501</v>
       </c>
       <c r="D22" s="6">
         <v>302318.0</v>
       </c>
       <c r="E22" s="4" t="s">
+        <v>501</v>
+      </c>
+      <c r="F22" s="4" t="s">
         <v>502</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>503</v>
       </c>
     </row>
     <row r="23" ht="18.75" customHeight="1">
       <c r="A23" s="10" t="s">
+        <v>503</v>
+      </c>
+      <c r="B23" s="4" t="s">
         <v>504</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="C23" s="5" t="s">
         <v>505</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>506</v>
       </c>
       <c r="D23" s="6">
         <v>319320.0</v>
       </c>
       <c r="E23" s="4" t="s">
+        <v>506</v>
+      </c>
+      <c r="F23" s="4" t="s">
         <v>507</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>508</v>
       </c>
     </row>
     <row r="24" ht="18.75" customHeight="1">
       <c r="A24" s="4" t="s">
+        <v>508</v>
+      </c>
+      <c r="B24" s="10" t="s">
         <v>509</v>
       </c>
-      <c r="B24" s="10" t="s">
+      <c r="C24" s="5" t="s">
         <v>510</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>511</v>
       </c>
       <c r="D24" s="6">
         <v>321334.0</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="F24" s="13"/>
     </row>
     <row r="25" ht="28.5" customHeight="1">
       <c r="A25" s="4" t="s">
+        <v>512</v>
+      </c>
+      <c r="B25" s="10" t="s">
         <v>513</v>
       </c>
-      <c r="B25" s="10" t="s">
+      <c r="C25" s="5" t="s">
         <v>514</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>515</v>
       </c>
       <c r="D25" s="6">
         <v>335474.0</v>
       </c>
       <c r="E25" s="4" t="s">
+        <v>515</v>
+      </c>
+      <c r="F25" s="4" t="s">
         <v>516</v>
-      </c>
-      <c r="F25" s="4" t="s">
-        <v>517</v>
       </c>
     </row>
     <row r="26" ht="64.5" customHeight="1">
       <c r="A26" s="10" t="s">
+        <v>517</v>
+      </c>
+      <c r="B26" s="10" t="s">
         <v>518</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="C26" s="5" t="s">
         <v>519</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>520</v>
       </c>
       <c r="D26" s="6">
         <v>475476.0</v>
       </c>
       <c r="E26" s="4" t="s">
+        <v>520</v>
+      </c>
+      <c r="F26" s="4" t="s">
         <v>521</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>522</v>
       </c>
     </row>
     <row r="27" ht="18.75" customHeight="1">
       <c r="A27" s="4" t="s">
+        <v>522</v>
+      </c>
+      <c r="B27" s="4" t="s">
         <v>523</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="C27" s="5" t="s">
         <v>524</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>525</v>
       </c>
       <c r="D27" s="6">
         <v>477490.0</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="F27" s="13"/>
     </row>
     <row r="28" ht="11.25" customHeight="1">
       <c r="A28" s="4" t="s">
+        <v>526</v>
+      </c>
+      <c r="B28" s="4" t="s">
         <v>527</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="C28" s="5" t="s">
         <v>528</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>529</v>
       </c>
       <c r="D28" s="6">
         <v>491630.0</v>
       </c>
       <c r="E28" s="4" t="s">
+        <v>529</v>
+      </c>
+      <c r="F28" s="4" t="s">
         <v>530</v>
-      </c>
-      <c r="F28" s="4" t="s">
-        <v>531</v>
       </c>
     </row>
     <row r="29" ht="18.75" customHeight="1">
       <c r="A29" s="4" t="s">
+        <v>531</v>
+      </c>
+      <c r="B29" s="4" t="s">
         <v>532</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="C29" s="5" t="s">
         <v>533</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>534</v>
       </c>
       <c r="D29" s="6">
         <v>631632.0</v>
       </c>
       <c r="E29" s="4" t="s">
+        <v>534</v>
+      </c>
+      <c r="F29" s="4" t="s">
         <v>535</v>
-      </c>
-      <c r="F29" s="4" t="s">
-        <v>536</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="4" t="s">
+        <v>536</v>
+      </c>
+      <c r="B30" s="4" t="s">
         <v>537</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="C30" s="5" t="s">
         <v>538</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>539</v>
       </c>
       <c r="D30" s="6">
         <v>633667.0</v>
       </c>
       <c r="E30" s="4" t="s">
+        <v>539</v>
+      </c>
+      <c r="F30" s="10" t="s">
         <v>540</v>
-      </c>
-      <c r="F30" s="10" t="s">
-        <v>541</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="4" t="s">
+        <v>541</v>
+      </c>
+      <c r="B31" s="4" t="s">
         <v>542</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="C31" s="5" t="s">
         <v>543</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>544</v>
       </c>
       <c r="D31" s="6">
         <v>668697.0</v>
       </c>
       <c r="E31" s="4" t="s">
+        <v>544</v>
+      </c>
+      <c r="F31" s="4" t="s">
         <v>545</v>
-      </c>
-      <c r="F31" s="4" t="s">
-        <v>546</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="4" t="s">
+        <v>546</v>
+      </c>
+      <c r="B32" s="4" t="s">
         <v>547</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="C32" s="5" t="s">
         <v>548</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>549</v>
       </c>
       <c r="D32" s="6">
         <v>698744.0</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="F32" s="14"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="4" t="s">
+        <v>550</v>
+      </c>
+      <c r="B33" s="4" t="s">
         <v>551</v>
       </c>
-      <c r="B33" s="4" t="s">
+      <c r="C33" s="5" t="s">
         <v>552</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>553</v>
       </c>
       <c r="D33" s="6">
         <v>745750.0</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="F33" s="13"/>
     </row>
@@ -15910,40 +15897,40 @@
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
       <c r="A1" s="1" t="s">
+        <v>554</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>555</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>556</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="17" t="s">
         <v>558</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="F1" s="1" t="s">
         <v>559</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>560</v>
       </c>
       <c r="G1" s="18"/>
     </row>
     <row r="2" ht="11.25" customHeight="1">
       <c r="A2" s="4" t="s">
+        <v>560</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>561</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="4" t="s">
         <v>562</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>563</v>
       </c>
       <c r="D2" s="6">
         <v>1001.0</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="F2" s="7">
         <v>2.0</v>
@@ -15951,147 +15938,147 @@
     </row>
     <row r="3" ht="18.75" customHeight="1">
       <c r="A3" s="4" t="s">
+        <v>564</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>565</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="C3" s="4" t="s">
         <v>566</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>567</v>
       </c>
       <c r="D3" s="6">
         <v>2036.0</v>
       </c>
       <c r="E3" s="19" t="s">
+        <v>567</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>568</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>569</v>
       </c>
     </row>
     <row r="4" ht="11.25" customHeight="1">
       <c r="A4" s="4" t="s">
+        <v>569</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>570</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C4" s="4" t="s">
         <v>571</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>572</v>
       </c>
       <c r="D4" s="6">
         <v>37086.0</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="F4" s="14"/>
     </row>
     <row r="5" ht="11.25" customHeight="1">
       <c r="A5" s="4" t="s">
+        <v>573</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>574</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>575</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>576</v>
       </c>
       <c r="D5" s="6">
         <v>87286.0</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="F5" s="14"/>
     </row>
     <row r="6" ht="11.25" customHeight="1">
       <c r="A6" s="4" t="s">
+        <v>577</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>578</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C6" s="4" t="s">
         <v>579</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>580</v>
       </c>
       <c r="D6" s="6">
         <v>287336.0</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="F6" s="14"/>
     </row>
     <row r="7" ht="11.25" customHeight="1">
       <c r="A7" s="4" t="s">
+        <v>581</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>582</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="C7" s="4" t="s">
         <v>583</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>584</v>
       </c>
       <c r="D7" s="6">
         <v>337536.0</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="F7" s="14"/>
     </row>
     <row r="8" ht="11.25" customHeight="1">
       <c r="A8" s="4" t="s">
+        <v>585</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>586</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="C8" s="4" t="s">
         <v>587</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>588</v>
       </c>
       <c r="D8" s="6">
         <v>537738.0</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="F8" s="14"/>
     </row>
     <row r="9" ht="11.25" customHeight="1">
       <c r="A9" s="4" t="s">
+        <v>589</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>590</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="C9" s="4" t="s">
         <v>591</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>592</v>
       </c>
       <c r="D9" s="6">
         <v>739744.0</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="F9" s="13"/>
     </row>
     <row r="10" ht="27.75" customHeight="1">
       <c r="A10" s="4" t="s">
+        <v>593</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>594</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="C10" s="4" t="s">
         <v>595</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>596</v>
       </c>
       <c r="D10" s="6">
         <v>745750.0</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="F10" s="13"/>
     </row>
@@ -17100,8 +17087,8 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A13:H13"/>
     <mergeCell ref="A14:H14"/>
-    <mergeCell ref="A13:H13"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
@@ -17129,40 +17116,40 @@
   <sheetData>
     <row r="1" ht="17.25" customHeight="1">
       <c r="A1" s="1" t="s">
+        <v>597</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>598</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>599</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>600</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="17" t="s">
         <v>601</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="F1" s="1" t="s">
         <v>602</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>603</v>
       </c>
       <c r="G1" s="18"/>
     </row>
     <row r="2" ht="27.0" customHeight="1">
       <c r="A2" s="4" t="s">
+        <v>603</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>604</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>605</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>606</v>
       </c>
       <c r="D2" s="6">
         <v>1001.0</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="F2" s="7">
         <v>3.0</v>
@@ -17170,155 +17157,155 @@
     </row>
     <row r="3" ht="11.25" customHeight="1">
       <c r="A3" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>608</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>609</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>610</v>
       </c>
       <c r="D3" s="6">
         <v>2078.0</v>
       </c>
       <c r="E3" s="19" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="F3" s="14"/>
     </row>
     <row r="4" ht="18.75" customHeight="1">
       <c r="A4" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>612</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>613</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>614</v>
       </c>
       <c r="D4" s="6">
         <v>79080.0</v>
       </c>
       <c r="E4" s="19" t="s">
+        <v>614</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>615</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>616</v>
       </c>
     </row>
     <row r="5" ht="18.75" customHeight="1">
       <c r="A5" s="4" t="s">
+        <v>616</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>617</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>618</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>619</v>
       </c>
       <c r="D5" s="6">
         <v>81088.0</v>
       </c>
       <c r="E5" s="19" t="s">
+        <v>619</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>620</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>621</v>
       </c>
     </row>
     <row r="6" ht="18.75" customHeight="1">
       <c r="A6" s="4" t="s">
+        <v>621</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>622</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>623</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>624</v>
       </c>
       <c r="D6" s="6">
         <v>89123.0</v>
       </c>
       <c r="E6" s="19" t="s">
+        <v>624</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>625</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>626</v>
       </c>
     </row>
     <row r="7" ht="11.25" customHeight="1">
       <c r="A7" s="4" t="s">
+        <v>626</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>627</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>628</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>629</v>
       </c>
       <c r="D7" s="6">
         <v>124623.0</v>
       </c>
       <c r="E7" s="19" t="s">
+        <v>629</v>
+      </c>
+      <c r="F7" s="4" t="s">
         <v>630</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>631</v>
       </c>
     </row>
     <row r="8" ht="18.0" customHeight="1">
       <c r="A8" s="4" t="s">
+        <v>631</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>632</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>633</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>634</v>
       </c>
       <c r="D8" s="6">
         <v>624700.0</v>
       </c>
       <c r="E8" s="19" t="s">
+        <v>634</v>
+      </c>
+      <c r="F8" s="10" t="s">
         <v>635</v>
-      </c>
-      <c r="F8" s="10" t="s">
-        <v>636</v>
       </c>
     </row>
     <row r="9" ht="11.25" customHeight="1">
       <c r="A9" s="4" t="s">
+        <v>636</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>637</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>638</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>639</v>
       </c>
       <c r="D9" s="6">
         <v>701744.0</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="F9" s="14"/>
     </row>
     <row r="10" ht="18.75" customHeight="1">
       <c r="A10" s="4" t="s">
+        <v>640</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>641</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="C10" s="5" t="s">
         <v>642</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>643</v>
       </c>
       <c r="D10" s="6">
         <v>745750.0</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="F10" s="13"/>
     </row>
@@ -18329,39 +18316,39 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
+        <v>644</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>645</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>646</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>647</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="17" t="s">
         <v>648</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="F1" s="1" t="s">
         <v>649</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>650</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="s">
+        <v>650</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>651</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>652</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>653</v>
       </c>
       <c r="D2" s="6">
         <v>1001.0</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="F2" s="7">
         <v>4.0</v>
@@ -18369,120 +18356,120 @@
     </row>
     <row r="3">
       <c r="A3" s="4" t="s">
+        <v>654</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>655</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>656</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>657</v>
       </c>
       <c r="D3" s="6">
         <v>2078.0</v>
       </c>
       <c r="E3" s="19" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="F3" s="14"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="s">
+        <v>658</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>659</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>660</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>661</v>
       </c>
       <c r="D4" s="6">
         <v>79080.0</v>
       </c>
       <c r="E4" s="19" t="s">
+        <v>661</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>662</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>663</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="s">
+        <v>663</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>664</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>665</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>666</v>
       </c>
       <c r="D5" s="6">
         <v>81088.0</v>
       </c>
       <c r="E5" s="19" t="s">
+        <v>666</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>667</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>668</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="s">
+        <v>668</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>669</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>670</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>671</v>
       </c>
       <c r="D6" s="6">
         <v>89123.0</v>
       </c>
       <c r="E6" s="19" t="s">
+        <v>671</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>672</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>673</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="s">
+        <v>673</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>674</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>675</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>676</v>
       </c>
       <c r="D7" s="6">
         <v>124623.0</v>
       </c>
       <c r="E7" s="19" t="s">
+        <v>676</v>
+      </c>
+      <c r="F7" s="4" t="s">
         <v>677</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>678</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="s">
+        <v>678</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>679</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>680</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>681</v>
       </c>
       <c r="D8" s="6">
         <v>624700.0</v>
       </c>
       <c r="E8" s="19" t="s">
+        <v>681</v>
+      </c>
+      <c r="F8" s="4" t="s">
         <v>682</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>683</v>
       </c>
     </row>
     <row r="9">
@@ -18490,44 +18477,44 @@
       <c r="B9" s="13"/>
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
-      <c r="E9" s="29"/>
+      <c r="E9" s="31"/>
       <c r="F9" s="4" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="s">
+        <v>684</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>685</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="C10" s="4" t="s">
         <v>686</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>687</v>
       </c>
       <c r="D10" s="6">
         <v>701744.0</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="F10" s="14"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="s">
+        <v>688</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>689</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="C11" s="4" t="s">
         <v>690</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>691</v>
       </c>
       <c r="D11" s="6">
         <v>745750.0</v>
       </c>
       <c r="E11" s="19" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="F11" s="13"/>
     </row>

</xml_diff>